<commit_message>
Stack creation debug: - one article can now fill mutliple stacks of one pallet (before, Iteration was interupted after first filled stack)
</commit_message>
<xml_diff>
--- a/Infeed_Test-michar.xlsx
+++ b/Infeed_Test-michar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gatmichar\Documents\fruit_salad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7DE020C6-23E3-40B1-8B27-ABB0C00D9E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA922F5F-5034-4416-8721-0673FD7837F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14310" yWindow="-21600" windowWidth="19410" windowHeight="20985" xr2:uid="{A3660F10-FBFE-4C97-B64C-95DC2948507A}"/>
+    <workbookView xWindow="-4890" yWindow="-21600" windowWidth="19410" windowHeight="20985" xr2:uid="{A3660F10-FBFE-4C97-B64C-95DC2948507A}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t>IN-ID</t>
   </si>
@@ -62,28 +62,10 @@
     <t>CT190</t>
   </si>
   <si>
-    <t>763345</t>
-  </si>
-  <si>
-    <t>FINOCCHI</t>
-  </si>
-  <si>
     <t>763164</t>
   </si>
   <si>
     <t>CAROTE NAT RESIDUO ZERO</t>
-  </si>
-  <si>
-    <t>753055</t>
-  </si>
-  <si>
-    <t>CAVOLFIORE BIO</t>
-  </si>
-  <si>
-    <t>761123</t>
-  </si>
-  <si>
-    <t>BANANE NATURAMA CTM</t>
   </si>
 </sst>
 </file>
@@ -138,11 +120,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -477,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A799C489-FE8B-4633-98E7-579E3BB1DAD9}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
@@ -505,106 +486,41 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2">
         <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="2">
-        <v>14</v>
+      <c r="E3">
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="2">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="2">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="2">
-        <v>53</v>
-      </c>
+      <c r="B4" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Improved Print-Statements: - more often article_code included for easier trackability - separated sections for Pallets, storage, Reservation activity in the terminal (better readability)
</commit_message>
<xml_diff>
--- a/Infeed_Test-michar.xlsx
+++ b/Infeed_Test-michar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gatmichar\Documents\fruit_salad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA922F5F-5034-4416-8721-0673FD7837F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B6A813-B553-4696-B5A2-23C319E26FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-4890" yWindow="-21600" windowWidth="19410" windowHeight="20985" xr2:uid="{A3660F10-FBFE-4C97-B64C-95DC2948507A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="16">
   <si>
     <t>IN-ID</t>
   </si>
@@ -62,10 +62,28 @@
     <t>CT190</t>
   </si>
   <si>
+    <t>763345</t>
+  </si>
+  <si>
+    <t>FINOCCHI</t>
+  </si>
+  <si>
     <t>763164</t>
   </si>
   <si>
     <t>CAROTE NAT RESIDUO ZERO</t>
+  </si>
+  <si>
+    <t>753055</t>
+  </si>
+  <si>
+    <t>CAVOLFIORE BIO</t>
+  </si>
+  <si>
+    <t>761123</t>
+  </si>
+  <si>
+    <t>BANANE NATURAMA CTM</t>
   </si>
 </sst>
 </file>
@@ -458,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A799C489-FE8B-4633-98E7-579E3BB1DAD9}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
@@ -516,11 +534,76 @@
         <v>7</v>
       </c>
       <c r="E3">
-        <v>30</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="2"/>
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7">
+        <v>53</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Debug of diff. crate Family: - if crate Family is different and first Family has an unfinished stack, the stack is cleared and filled with the second crate family
</commit_message>
<xml_diff>
--- a/Infeed_Test-michar.xlsx
+++ b/Infeed_Test-michar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gatmichar\Documents\fruit_salad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A22BB95-1335-490B-892A-0980AF0B02E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3D6A242-D11F-40E3-9D0C-7D74601E2605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-4890" yWindow="-21600" windowWidth="19410" windowHeight="20985" xr2:uid="{A3660F10-FBFE-4C97-B64C-95DC2948507A}"/>
   </bookViews>
@@ -86,7 +86,7 @@
     <t>BANANE NATURAMA CTM</t>
   </si>
   <si>
-    <t>ABC</t>
+    <t>IFCO6420</t>
   </si>
 </sst>
 </file>
@@ -535,16 +535,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3">
-        <v>14</v>
+        <v>10</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="3">
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -586,16 +586,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="3">
-        <v>13</v>
+      <c r="E6">
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -609,7 +609,7 @@
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E7">
         <v>53</v>

</xml_diff>

<commit_message>
Open Points Outfeed & Test Cases: - open Points/Questions for outfeed logic are listed at very Bottom of outfeed file - Excel with test cases added in file structure. should be maintained for structured Regression testing - in the structure of "stack_contents", now, the article code is also included (for printing article code for each palletized crate)
</commit_message>
<xml_diff>
--- a/Infeed_Test-michar.xlsx
+++ b/Infeed_Test-michar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gatmichar\Documents\fruit_salad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3D6A242-D11F-40E3-9D0C-7D74601E2605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A6750B-05B5-4306-9A58-EEFB8C69FFF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-4890" yWindow="-21600" windowWidth="19410" windowHeight="20985" xr2:uid="{A3660F10-FBFE-4C97-B64C-95DC2948507A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
   <si>
     <t>IN-ID</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>IFCO6420</t>
+  </si>
+  <si>
+    <t>CT250</t>
   </si>
 </sst>
 </file>
@@ -110,18 +113,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -147,11 +144,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -486,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A799C489-FE8B-4633-98E7-579E3BB1DAD9}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
@@ -496,7 +492,7 @@
     <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -513,45 +509,47 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E2">
+        <v>8</v>
+      </c>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="3">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E3">
+        <v>18</v>
+      </c>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>14</v>
       </c>
       <c r="C4" t="s">
@@ -561,59 +559,142 @@
         <v>7</v>
       </c>
       <c r="E4">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>14</v>
+      <c r="B5" t="s">
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
       </c>
       <c r="E5">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
       </c>
       <c r="E6">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
+      <c r="B7" t="s">
+        <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="E7">
-        <v>53</v>
-      </c>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>